<commit_message>
Update biography by adding achievements for some players and teams.
</commit_message>
<xml_diff>
--- a/excel/player_personal_awards.xlsx
+++ b/excel/player_personal_awards.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="38">
   <si>
     <t>id</t>
   </si>
@@ -98,6 +98,33 @@
   </si>
   <si>
     <t>opm_10</t>
+  </si>
+  <si>
+    <t>tfs10MVPAFC2025</t>
+  </si>
+  <si>
+    <t>tfs_10</t>
+  </si>
+  <si>
+    <t>tfs</t>
+  </si>
+  <si>
+    <t>tfs14PMAFC2025</t>
+  </si>
+  <si>
+    <t>tfs_14</t>
+  </si>
+  <si>
+    <t>tfs10GBAFC2025</t>
+  </si>
+  <si>
+    <t>dbz1BGKAFC2025</t>
+  </si>
+  <si>
+    <t>dbz_1</t>
+  </si>
+  <si>
+    <t>dbz</t>
   </si>
 </sst>
 </file>
@@ -1454,39 +1481,87 @@
       <c r="G8" s="9"/>
     </row>
     <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
+      <c r="A9" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s" s="7">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s" s="7">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s" s="7">
+        <v>31</v>
+      </c>
+      <c r="F9" s="8">
+        <v>2025</v>
+      </c>
       <c r="G9" s="9"/>
     </row>
     <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
+      <c r="A10" t="s" s="7">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s" s="7">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s" s="7">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s" s="7">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s" s="7">
+        <v>31</v>
+      </c>
+      <c r="F10" s="8">
+        <v>2025</v>
+      </c>
       <c r="G10" s="9"/>
     </row>
     <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
+      <c r="A11" t="s" s="7">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s" s="7">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s" s="7">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s" s="7">
+        <v>31</v>
+      </c>
+      <c r="F11" s="8">
+        <v>2025</v>
+      </c>
       <c r="G11" s="9"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+      <c r="A12" t="s" s="7">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s" s="7">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="D12" t="s" s="7">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s" s="7">
+        <v>37</v>
+      </c>
+      <c r="F12" s="8">
+        <v>2025</v>
+      </c>
       <c r="G12" s="9"/>
     </row>
     <row r="13" ht="20.05" customHeight="1">

</xml_diff>